<commit_message>
Update macroeconomic indicators documentation to reflect adjustments in indicator classifications
- Revised the classification of `LPR_1Y` and removed `RRR_LARGE_FIN_INST` from the "财政、民生与政策工具" section, consolidating it under "货币、信用与利率" to better represent its role in financial conditions.
- Updated the total count of independent indicators in the documentation to ensure accuracy.
- Enhanced clarity in the notes regarding the categorization of indicators, reflecting the latest adjustments in the dataset.
</commit_message>
<xml_diff>
--- a/docs/智能投顾数据.xlsx
+++ b/docs/智能投顾数据.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="15240" activeTab="3"/>
+    <workbookView windowWidth="30460" windowHeight="18180"/>
   </bookViews>
   <sheets>
     <sheet name="境内宏观" sheetId="1" r:id="rId1"/>
@@ -13,7 +13,7 @@
     <sheet name="行情展示" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">境内宏观!$A$1:$J$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">境内宏观!$A$1:$J$38</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">境外宏观!$A$1:$I$25</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">大类资产!$A$1:$J$68</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">行情展示!$A$1:$J$21</definedName>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1515" uniqueCount="338">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1492" uniqueCount="333">
   <si>
     <t>指标代码</t>
   </si>
@@ -161,15 +161,9 @@
     <t>出口金额:当月同比</t>
   </si>
   <si>
-    <t>与采购清单V3不一致：V3为"出口金额:累计同比"</t>
-  </si>
-  <si>
     <t>进口金额:当月同比</t>
   </si>
   <si>
-    <t>与采购清单V3不一致：V3为"进口金额:累计同比"</t>
-  </si>
-  <si>
     <t>城镇调查失业率</t>
   </si>
   <si>
@@ -299,336 +293,330 @@
     <t>EMM01430555</t>
   </si>
   <si>
+    <t>商品房销售额:住宅:累计同比</t>
+  </si>
+  <si>
+    <t>EMM00877640</t>
+  </si>
+  <si>
+    <t>AA级信用债收益率（3年）</t>
+  </si>
+  <si>
+    <t>信用</t>
+  </si>
+  <si>
+    <t>E1000469</t>
+  </si>
+  <si>
+    <t>GDP（年度环比）</t>
+  </si>
+  <si>
+    <t>经济增长</t>
+  </si>
+  <si>
+    <t>零售销售</t>
+  </si>
+  <si>
+    <t>耐用品订单</t>
+  </si>
+  <si>
+    <t>投资</t>
+  </si>
+  <si>
+    <t>成屋/新屋销售数量/价格</t>
+  </si>
+  <si>
+    <t>地产</t>
+  </si>
+  <si>
+    <t>新屋开工/施工/竣工</t>
+  </si>
+  <si>
+    <t>失业率</t>
+  </si>
+  <si>
+    <t>劳动参与率</t>
+  </si>
+  <si>
+    <t>非农新增就业</t>
+  </si>
+  <si>
+    <t>薪资</t>
+  </si>
+  <si>
+    <t>ADP就业</t>
+  </si>
+  <si>
+    <t>首次申请失业金人数</t>
+  </si>
+  <si>
+    <t>周度</t>
+  </si>
+  <si>
+    <t>续请失业金人数</t>
+  </si>
+  <si>
+    <t>ISM制造业PMI</t>
+  </si>
+  <si>
+    <t>ISM服务业PMI</t>
+  </si>
+  <si>
+    <t>Markit PMI</t>
+  </si>
+  <si>
+    <t>消费者信心指数</t>
+  </si>
+  <si>
+    <t>CPI</t>
+  </si>
+  <si>
+    <t>核心CPI</t>
+  </si>
+  <si>
+    <t>PCE</t>
+  </si>
+  <si>
+    <t>核心PCE</t>
+  </si>
+  <si>
+    <t>PPI</t>
+  </si>
+  <si>
+    <t>核心PPI</t>
+  </si>
+  <si>
+    <t>居民可支配收入</t>
+  </si>
+  <si>
+    <t>消费</t>
+  </si>
+  <si>
+    <t>实际消费</t>
+  </si>
+  <si>
+    <t>资产类别</t>
+  </si>
+  <si>
+    <t>定位</t>
+  </si>
+  <si>
+    <t>港股</t>
+  </si>
+  <si>
+    <t>G8326461</t>
+  </si>
+  <si>
+    <t>港交所:恒生指数:平均市盈率</t>
+  </si>
+  <si>
+    <t>月</t>
+  </si>
+  <si>
+    <t>L9882961</t>
+  </si>
+  <si>
+    <t>恒生科技指数</t>
+  </si>
+  <si>
+    <t>日</t>
+  </si>
+  <si>
+    <t>G0001693</t>
+  </si>
+  <si>
+    <t>恒生指数</t>
+  </si>
+  <si>
+    <t>M0058006</t>
+  </si>
+  <si>
+    <t>恒生AH股溢价指数</t>
+  </si>
+  <si>
+    <t>V5026793</t>
+  </si>
+  <si>
+    <t>市盈率:恒生科技指数</t>
+  </si>
+  <si>
+    <t>汇率</t>
+  </si>
+  <si>
+    <t>M0000271</t>
+  </si>
+  <si>
+    <t>美元指数</t>
+  </si>
+  <si>
+    <t>M0000185</t>
+  </si>
+  <si>
+    <t>中间价:美元兑人民币</t>
+  </si>
+  <si>
+    <t>EMM00058124</t>
+  </si>
+  <si>
+    <t>M0067858</t>
+  </si>
+  <si>
+    <t>CFETS:即期汇率:100日元兑人民币</t>
+  </si>
+  <si>
+    <t>M0067857</t>
+  </si>
+  <si>
+    <t>CFETS:即期汇率:港元兑人民币</t>
+  </si>
+  <si>
+    <t>M0067855</t>
+  </si>
+  <si>
+    <t>CFETS:即期汇率:美元兑人民币</t>
+  </si>
+  <si>
+    <t>M0067856</t>
+  </si>
+  <si>
+    <t>CFETS:即期汇率:欧元兑人民币</t>
+  </si>
+  <si>
+    <t>M0327998</t>
+  </si>
+  <si>
+    <t>CFETS:即期汇率:人民币兑韩元</t>
+  </si>
+  <si>
+    <t>M0067859</t>
+  </si>
+  <si>
+    <t>CFETS:即期汇率:英镑兑人民币</t>
+  </si>
+  <si>
+    <t>M0325601</t>
+  </si>
+  <si>
+    <t>CFETS人民币汇率指数</t>
+  </si>
+  <si>
+    <t>周</t>
+  </si>
+  <si>
+    <t>境内债券&amp;利率</t>
+  </si>
+  <si>
+    <t>S0213048</t>
+  </si>
+  <si>
+    <t>期货结算价(活跃合约):国债期货:10年期</t>
+  </si>
+  <si>
+    <t>M0330936</t>
+  </si>
+  <si>
+    <t>期货结算价(活跃合约):国债期货:2年期</t>
+  </si>
+  <si>
+    <t>M0096849</t>
+  </si>
+  <si>
+    <t>期货收盘价(活跃合约):国债期货:5年</t>
+  </si>
+  <si>
+    <t>M0096870</t>
+  </si>
+  <si>
+    <t>中国:贷款市场报价利率(LPR):1年</t>
+  </si>
+  <si>
+    <t>M0017153</t>
+  </si>
+  <si>
+    <t>中国:回购定盘利率:7天(FR007)</t>
+  </si>
+  <si>
+    <t>M0329545</t>
+  </si>
+  <si>
+    <t>中国:利率:中期借贷便利(MLF):1年</t>
+  </si>
+  <si>
+    <t>M0041371</t>
+  </si>
+  <si>
+    <t>中国:逆回购利率:7天</t>
+  </si>
+  <si>
+    <t>S0059749</t>
+  </si>
+  <si>
+    <t>中债国债到期收益率:10年</t>
+  </si>
+  <si>
+    <t>E1000180</t>
+  </si>
+  <si>
+    <t>S0059744</t>
+  </si>
+  <si>
+    <t>中债国债到期收益率:1年</t>
+  </si>
+  <si>
+    <t>E1000172</t>
+  </si>
+  <si>
+    <t>S0059752</t>
+  </si>
+  <si>
+    <t>中债国债到期收益率:30年</t>
+  </si>
+  <si>
+    <t>S0059741</t>
+  </si>
+  <si>
+    <t>中债国债到期收益率:3个月</t>
+  </si>
+  <si>
+    <t>S0059747</t>
+  </si>
+  <si>
+    <t>中债国债到期收益率:5年</t>
+  </si>
+  <si>
+    <t>M1010885</t>
+  </si>
+  <si>
+    <t>中债商业银行同业存单到期收益率(AAA):1年</t>
+  </si>
+  <si>
+    <t>M0265754</t>
+  </si>
+  <si>
+    <t>中债信用债总指数</t>
+  </si>
+  <si>
+    <t>M0265843</t>
+  </si>
+  <si>
+    <t>中债长期债券净价指数</t>
+  </si>
+  <si>
+    <t>M0265842</t>
+  </si>
+  <si>
+    <t>中债中短期债券净价指数</t>
+  </si>
+  <si>
+    <t>M1006337</t>
+  </si>
+  <si>
     <t>DR007</t>
   </si>
   <si>
     <t>E1300004</t>
   </si>
   <si>
-    <t>中国:人民币存款准备金率:大型存款类金融机构(月)</t>
-  </si>
-  <si>
-    <t>EMM01280574</t>
-  </si>
-  <si>
-    <t>商品房销售额:住宅:累计同比</t>
-  </si>
-  <si>
-    <t>EMM00877640</t>
-  </si>
-  <si>
-    <t>AA级信用债收益率（3年）</t>
-  </si>
-  <si>
-    <t>信用</t>
-  </si>
-  <si>
-    <t>E1000469</t>
-  </si>
-  <si>
-    <t>GDP（年度环比）</t>
-  </si>
-  <si>
-    <t>经济增长</t>
-  </si>
-  <si>
-    <t>零售销售</t>
-  </si>
-  <si>
-    <t>耐用品订单</t>
-  </si>
-  <si>
-    <t>投资</t>
-  </si>
-  <si>
-    <t>成屋/新屋销售数量/价格</t>
-  </si>
-  <si>
-    <t>地产</t>
-  </si>
-  <si>
-    <t>新屋开工/施工/竣工</t>
-  </si>
-  <si>
-    <t>失业率</t>
-  </si>
-  <si>
-    <t>劳动参与率</t>
-  </si>
-  <si>
-    <t>非农新增就业</t>
-  </si>
-  <si>
-    <t>薪资</t>
-  </si>
-  <si>
-    <t>ADP就业</t>
-  </si>
-  <si>
-    <t>首次申请失业金人数</t>
-  </si>
-  <si>
-    <t>周度</t>
-  </si>
-  <si>
-    <t>续请失业金人数</t>
-  </si>
-  <si>
-    <t>ISM制造业PMI</t>
-  </si>
-  <si>
-    <t>ISM服务业PMI</t>
-  </si>
-  <si>
-    <t>Markit PMI</t>
-  </si>
-  <si>
-    <t>消费者信心指数</t>
-  </si>
-  <si>
-    <t>CPI</t>
-  </si>
-  <si>
-    <t>核心CPI</t>
-  </si>
-  <si>
-    <t>PCE</t>
-  </si>
-  <si>
-    <t>核心PCE</t>
-  </si>
-  <si>
-    <t>PPI</t>
-  </si>
-  <si>
-    <t>核心PPI</t>
-  </si>
-  <si>
-    <t>居民可支配收入</t>
-  </si>
-  <si>
-    <t>消费</t>
-  </si>
-  <si>
-    <t>实际消费</t>
-  </si>
-  <si>
-    <t>资产类别</t>
-  </si>
-  <si>
-    <t>定位</t>
-  </si>
-  <si>
-    <t>港股</t>
-  </si>
-  <si>
-    <t>G8326461</t>
-  </si>
-  <si>
-    <t>港交所:恒生指数:平均市盈率</t>
-  </si>
-  <si>
-    <t>月</t>
-  </si>
-  <si>
-    <t>L9882961</t>
-  </si>
-  <si>
-    <t>恒生科技指数</t>
-  </si>
-  <si>
-    <t>日</t>
-  </si>
-  <si>
-    <t>G0001693</t>
-  </si>
-  <si>
-    <t>恒生指数</t>
-  </si>
-  <si>
-    <t>M0058006</t>
-  </si>
-  <si>
-    <t>恒生AH股溢价指数</t>
-  </si>
-  <si>
-    <t>V5026793</t>
-  </si>
-  <si>
-    <t>市盈率:恒生科技指数</t>
-  </si>
-  <si>
-    <t>汇率</t>
-  </si>
-  <si>
-    <t>M0000271</t>
-  </si>
-  <si>
-    <t>美元指数</t>
-  </si>
-  <si>
-    <t>M0000185</t>
-  </si>
-  <si>
-    <t>中间价:美元兑人民币</t>
-  </si>
-  <si>
-    <t>EMM00058124</t>
-  </si>
-  <si>
-    <t>M0067858</t>
-  </si>
-  <si>
-    <t>CFETS:即期汇率:100日元兑人民币</t>
-  </si>
-  <si>
-    <t>M0067857</t>
-  </si>
-  <si>
-    <t>CFETS:即期汇率:港元兑人民币</t>
-  </si>
-  <si>
-    <t>M0067855</t>
-  </si>
-  <si>
-    <t>CFETS:即期汇率:美元兑人民币</t>
-  </si>
-  <si>
-    <t>M0067856</t>
-  </si>
-  <si>
-    <t>CFETS:即期汇率:欧元兑人民币</t>
-  </si>
-  <si>
-    <t>M0327998</t>
-  </si>
-  <si>
-    <t>CFETS:即期汇率:人民币兑韩元</t>
-  </si>
-  <si>
-    <t>M0067859</t>
-  </si>
-  <si>
-    <t>CFETS:即期汇率:英镑兑人民币</t>
-  </si>
-  <si>
-    <t>M0325601</t>
-  </si>
-  <si>
-    <t>CFETS人民币汇率指数</t>
-  </si>
-  <si>
-    <t>周</t>
-  </si>
-  <si>
-    <t>境内债券&amp;利率</t>
-  </si>
-  <si>
-    <t>S0213048</t>
-  </si>
-  <si>
-    <t>期货结算价(活跃合约):国债期货:10年期</t>
-  </si>
-  <si>
-    <t>M0330936</t>
-  </si>
-  <si>
-    <t>期货结算价(活跃合约):国债期货:2年期</t>
-  </si>
-  <si>
-    <t>M0096849</t>
-  </si>
-  <si>
-    <t>期货收盘价(活跃合约):国债期货:5年</t>
-  </si>
-  <si>
-    <t>M0096870</t>
-  </si>
-  <si>
-    <t>中国:贷款市场报价利率(LPR):1年</t>
-  </si>
-  <si>
-    <t>M0017153</t>
-  </si>
-  <si>
-    <t>中国:回购定盘利率:7天(FR007)</t>
-  </si>
-  <si>
-    <t>M0329545</t>
-  </si>
-  <si>
-    <t>中国:利率:中期借贷便利(MLF):1年</t>
-  </si>
-  <si>
-    <t>M0041371</t>
-  </si>
-  <si>
-    <t>中国:逆回购利率:7天</t>
-  </si>
-  <si>
-    <t>S0059749</t>
-  </si>
-  <si>
-    <t>中债国债到期收益率:10年</t>
-  </si>
-  <si>
-    <t>E1000180</t>
-  </si>
-  <si>
-    <t>S0059744</t>
-  </si>
-  <si>
-    <t>中债国债到期收益率:1年</t>
-  </si>
-  <si>
-    <t>E1000172</t>
-  </si>
-  <si>
-    <t>S0059752</t>
-  </si>
-  <si>
-    <t>中债国债到期收益率:30年</t>
-  </si>
-  <si>
-    <t>S0059741</t>
-  </si>
-  <si>
-    <t>中债国债到期收益率:3个月</t>
-  </si>
-  <si>
-    <t>S0059747</t>
-  </si>
-  <si>
-    <t>中债国债到期收益率:5年</t>
-  </si>
-  <si>
-    <t>M1010885</t>
-  </si>
-  <si>
-    <t>中债商业银行同业存单到期收益率(AAA):1年</t>
-  </si>
-  <si>
-    <t>M0265754</t>
-  </si>
-  <si>
-    <t>中债信用债总指数</t>
-  </si>
-  <si>
-    <t>M0265843</t>
-  </si>
-  <si>
-    <t>中债长期债券净价指数</t>
-  </si>
-  <si>
-    <t>M0265842</t>
-  </si>
-  <si>
-    <t>中债中短期债券净价指数</t>
-  </si>
-  <si>
-    <t>M1006337</t>
-  </si>
-  <si>
     <t>A股</t>
   </si>
   <si>
@@ -1047,19 +1035,6 @@
   </si>
   <si>
     <t>南华商品</t>
-  </si>
-  <si>
-    <r>
-      <t>确认是否可作为商品主腿，</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t>NHCI</t>
-    </r>
   </si>
 </sst>
 </file>
@@ -1072,7 +1047,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1096,13 +1071,6 @@
       <sz val="10"/>
       <name val="宋体-简"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <u/>
@@ -1579,28 +1547,31 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1609,118 +1580,115 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -2084,7 +2052,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:J40"/>
+  <dimension ref="A1:J38"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -2573,16 +2541,14 @@
       <c r="I15" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="J15" s="3" t="s">
-        <v>41</v>
-      </c>
+      <c r="J15" s="3"/>
     </row>
     <row r="16" spans="1:10">
       <c r="A16" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>12</v>
@@ -2605,16 +2571,14 @@
       <c r="I16" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="J16" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="J16" s="2"/>
     </row>
     <row r="17" spans="1:10">
       <c r="A17" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>12</v>
@@ -2632,10 +2596,10 @@
         <v>10</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="J17" s="3" t="s">
         <v>10</v>
@@ -2646,7 +2610,7 @@
         <v>10</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>12</v>
@@ -2664,10 +2628,10 @@
         <v>10</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="J18" s="2" t="s">
         <v>10</v>
@@ -2678,7 +2642,7 @@
         <v>10</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>12</v>
@@ -2696,10 +2660,10 @@
         <v>10</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="J19" s="3" t="s">
         <v>10</v>
@@ -2710,7 +2674,7 @@
         <v>10</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>12</v>
@@ -2728,10 +2692,10 @@
         <v>10</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="J20" s="2" t="s">
         <v>10</v>
@@ -2742,7 +2706,7 @@
         <v>10</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>12</v>
@@ -2760,10 +2724,10 @@
         <v>10</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="J21" s="3" t="s">
         <v>10</v>
@@ -2774,7 +2738,7 @@
         <v>10</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>12</v>
@@ -2792,10 +2756,10 @@
         <v>10</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="J22" s="2" t="s">
         <v>10</v>
@@ -2806,25 +2770,25 @@
         <v>10</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>12</v>
       </c>
       <c r="D23" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="H23" s="3" t="s">
         <v>60</v>
-      </c>
-      <c r="E23" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="F23" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G23" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="H23" s="3" t="s">
-        <v>62</v>
       </c>
       <c r="I23" s="3" t="s">
         <v>10</v>
@@ -2838,7 +2802,7 @@
         <v>10</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>12</v>
@@ -2856,7 +2820,7 @@
         <v>10</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I24" s="2" t="s">
         <v>10</v>
@@ -2870,7 +2834,7 @@
         <v>10</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>12</v>
@@ -2888,10 +2852,10 @@
         <v>10</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I25" s="3" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="J25" s="3" t="s">
         <v>10</v>
@@ -2902,7 +2866,7 @@
         <v>10</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>12</v>
@@ -2920,7 +2884,7 @@
         <v>10</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I26" s="2" t="s">
         <v>10</v>
@@ -2934,7 +2898,7 @@
         <v>10</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C27" s="3" t="s">
         <v>12</v>
@@ -2952,7 +2916,7 @@
         <v>10</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I27" s="3" t="s">
         <v>10</v>
@@ -2966,25 +2930,25 @@
         <v>10</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D28" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H28" s="2" t="s">
         <v>69</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="F28" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G28" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="H28" s="2" t="s">
-        <v>71</v>
       </c>
       <c r="I28" s="2" t="s">
         <v>10</v>
@@ -2998,7 +2962,7 @@
         <v>10</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C29" s="3" t="s">
         <v>12</v>
@@ -3016,7 +2980,7 @@
         <v>10</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="I29" s="3" t="s">
         <v>10</v>
@@ -3030,7 +2994,7 @@
         <v>10</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>12</v>
@@ -3048,10 +3012,10 @@
         <v>10</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="J30" s="2" t="s">
         <v>10</v>
@@ -3062,7 +3026,7 @@
         <v>10</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C31" s="3" t="s">
         <v>12</v>
@@ -3080,7 +3044,7 @@
         <v>10</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="I31" s="3" t="s">
         <v>10</v>
@@ -3094,7 +3058,7 @@
         <v>10</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>12</v>
@@ -3115,10 +3079,10 @@
         <v>29</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J32" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="33" spans="1:10">
@@ -3126,7 +3090,7 @@
         <v>10</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C33" s="3" t="s">
         <v>12</v>
@@ -3147,10 +3111,10 @@
         <v>29</v>
       </c>
       <c r="I33" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="J33" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="34" spans="1:10">
@@ -3158,7 +3122,7 @@
         <v>10</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>12</v>
@@ -3179,10 +3143,10 @@
         <v>29</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="J34" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="35" spans="1:10">
@@ -3190,7 +3154,7 @@
         <v>10</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C35" s="3" t="s">
         <v>12</v>
@@ -3208,13 +3172,13 @@
         <v>10</v>
       </c>
       <c r="H35" s="3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I35" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="J35" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="36" spans="1:10">
@@ -3222,31 +3186,31 @@
         <v>10</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D36" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H36" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E36" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="F36" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G36" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="H36" s="2" t="s">
-        <v>62</v>
-      </c>
       <c r="I36" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J36" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="37" spans="1:10">
@@ -3254,16 +3218,16 @@
         <v>10</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C37" s="3" t="s">
         <v>12</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>69</v>
+        <v>18</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>70</v>
+        <v>19</v>
       </c>
       <c r="F37" s="3" t="s">
         <v>10</v>
@@ -3272,13 +3236,13 @@
         <v>10</v>
       </c>
       <c r="H37" s="3" t="s">
-        <v>71</v>
+        <v>29</v>
       </c>
       <c r="I37" s="3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="J37" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="38" spans="1:10">
@@ -3286,16 +3250,16 @@
         <v>10</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>18</v>
+        <v>67</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>19</v>
+        <v>68</v>
       </c>
       <c r="F38" s="2" t="s">
         <v>10</v>
@@ -3304,81 +3268,17 @@
         <v>10</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>71</v>
+        <v>88</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="J38" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10">
-      <c r="A39" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B39" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="C39" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D39" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E39" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="F39" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G39" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="H39" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="I39" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="J39" s="3" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10">
-      <c r="A40" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="E40" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="F40" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G40" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="H40" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="I40" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="J40" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:J40" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:J38" etc:filterBottomFollowUsedRange="0">
     <extLst/>
   </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3435,7 +3335,7 @@
         <v>10</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>12</v>
@@ -3453,7 +3353,7 @@
         <v>10</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>10</v>
@@ -3464,7 +3364,7 @@
         <v>10</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>12</v>
@@ -3482,7 +3382,7 @@
         <v>10</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="I3" s="3" t="s">
         <v>10</v>
@@ -3493,7 +3393,7 @@
         <v>10</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>12</v>
@@ -3511,7 +3411,7 @@
         <v>10</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>10</v>
@@ -3522,7 +3422,7 @@
         <v>10</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>12</v>
@@ -3540,7 +3440,7 @@
         <v>10</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="I5" s="3" t="s">
         <v>10</v>
@@ -3551,7 +3451,7 @@
         <v>10</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>12</v>
@@ -3569,7 +3469,7 @@
         <v>10</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>10</v>
@@ -3580,7 +3480,7 @@
         <v>10</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>12</v>
@@ -3598,7 +3498,7 @@
         <v>10</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I7" s="3" t="s">
         <v>10</v>
@@ -3609,7 +3509,7 @@
         <v>10</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>12</v>
@@ -3627,7 +3527,7 @@
         <v>10</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>10</v>
@@ -3638,7 +3538,7 @@
         <v>10</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>12</v>
@@ -3656,7 +3556,7 @@
         <v>10</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I9" s="3" t="s">
         <v>10</v>
@@ -3667,7 +3567,7 @@
         <v>10</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>12</v>
@@ -3685,7 +3585,7 @@
         <v>10</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>10</v>
@@ -3696,7 +3596,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>12</v>
@@ -3714,7 +3614,7 @@
         <v>10</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I11" s="3" t="s">
         <v>10</v>
@@ -3725,16 +3625,16 @@
         <v>10</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>10</v>
@@ -3743,7 +3643,7 @@
         <v>10</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>10</v>
@@ -3754,16 +3654,16 @@
         <v>10</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="F13" s="3" t="s">
         <v>10</v>
@@ -3772,7 +3672,7 @@
         <v>10</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I13" s="3" t="s">
         <v>10</v>
@@ -3783,7 +3683,7 @@
         <v>10</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>12</v>
@@ -3812,7 +3712,7 @@
         <v>10</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>12</v>
@@ -3841,7 +3741,7 @@
         <v>10</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>12</v>
@@ -3870,7 +3770,7 @@
         <v>10</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>12</v>
@@ -3899,7 +3799,7 @@
         <v>10</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>12</v>
@@ -3917,7 +3817,7 @@
         <v>10</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="I18" s="2" t="s">
         <v>10</v>
@@ -3928,7 +3828,7 @@
         <v>10</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>12</v>
@@ -3946,7 +3846,7 @@
         <v>10</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="I19" s="3" t="s">
         <v>10</v>
@@ -3957,7 +3857,7 @@
         <v>10</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>12</v>
@@ -3975,7 +3875,7 @@
         <v>10</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="I20" s="2" t="s">
         <v>10</v>
@@ -3986,7 +3886,7 @@
         <v>10</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>12</v>
@@ -4004,7 +3904,7 @@
         <v>10</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="I21" s="3" t="s">
         <v>10</v>
@@ -4015,7 +3915,7 @@
         <v>10</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>12</v>
@@ -4033,7 +3933,7 @@
         <v>10</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="I22" s="2" t="s">
         <v>10</v>
@@ -4044,7 +3944,7 @@
         <v>10</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>12</v>
@@ -4062,7 +3962,7 @@
         <v>10</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="I23" s="3" t="s">
         <v>10</v>
@@ -4073,7 +3973,7 @@
         <v>10</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>12</v>
@@ -4091,7 +3991,7 @@
         <v>10</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="I24" s="2" t="s">
         <v>10</v>
@@ -4102,7 +4002,7 @@
         <v>10</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>12</v>
@@ -4120,7 +4020,7 @@
         <v>10</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="I25" s="3" t="s">
         <v>10</v>
@@ -4153,7 +4053,7 @@
   <sheetData>
     <row r="1" ht="17" spans="1:10">
       <c r="A1" s="1" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -4174,7 +4074,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>8</v>
@@ -4185,22 +4085,22 @@
     </row>
     <row r="2" spans="1:10">
       <c r="A2" s="2" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>10</v>
@@ -4217,22 +4117,22 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" s="3" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G3" s="3" t="s">
         <v>10</v>
@@ -4249,22 +4149,22 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" s="2" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>10</v>
@@ -4281,22 +4181,22 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="3" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G5" s="3" t="s">
         <v>10</v>
@@ -4313,22 +4213,22 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" s="2" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>10</v>
@@ -4345,22 +4245,22 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" s="3" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G7" s="3" t="s">
         <v>10</v>
@@ -4377,22 +4277,22 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="2" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>10</v>
@@ -4401,7 +4301,7 @@
         <v>10</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="J8" s="2" t="s">
         <v>10</v>
@@ -4409,22 +4309,22 @@
     </row>
     <row r="9" spans="1:10">
       <c r="A9" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="B9" s="3" t="s">
-        <v>146</v>
-      </c>
       <c r="C9" s="3" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G9" s="3" t="s">
         <v>10</v>
@@ -4441,22 +4341,22 @@
     </row>
     <row r="10" spans="1:10">
       <c r="A10" s="2" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>10</v>
@@ -4473,22 +4373,22 @@
     </row>
     <row r="11" spans="1:10">
       <c r="A11" s="3" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G11" s="3" t="s">
         <v>10</v>
@@ -4505,22 +4405,22 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="2" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>10</v>
@@ -4537,22 +4437,22 @@
     </row>
     <row r="13" spans="1:10">
       <c r="A13" s="3" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="D13" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G13" s="3" t="s">
         <v>10</v>
@@ -4569,22 +4469,22 @@
     </row>
     <row r="14" spans="1:10">
       <c r="A14" s="2" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>10</v>
@@ -4601,22 +4501,22 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" s="3" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="G15" s="3" t="s">
         <v>10</v>
@@ -4633,22 +4533,22 @@
     </row>
     <row r="16" spans="1:10">
       <c r="A16" s="2" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>10</v>
@@ -4665,22 +4565,22 @@
     </row>
     <row r="17" spans="1:10">
       <c r="A17" s="3" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G17" s="3" t="s">
         <v>10</v>
@@ -4697,22 +4597,22 @@
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="B18" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="D18" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>10</v>
@@ -4729,22 +4629,22 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" s="3" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="D19" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G19" s="3" t="s">
         <v>10</v>
@@ -4761,22 +4661,22 @@
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="2" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>10</v>
@@ -4793,22 +4693,22 @@
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="3" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="D21" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G21" s="3" t="s">
         <v>10</v>
@@ -4825,22 +4725,22 @@
     </row>
     <row r="22" spans="1:10">
       <c r="A22" s="2" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G22" s="2" t="s">
         <v>10</v>
@@ -4857,22 +4757,22 @@
     </row>
     <row r="23" spans="1:10">
       <c r="A23" s="3" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="D23" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G23" s="3" t="s">
         <v>10</v>
@@ -4881,7 +4781,7 @@
         <v>10</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="J23" s="3" t="s">
         <v>10</v>
@@ -4889,22 +4789,22 @@
     </row>
     <row r="24" spans="1:10">
       <c r="A24" s="2" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>10</v>
@@ -4913,7 +4813,7 @@
         <v>10</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="J24" s="2" t="s">
         <v>10</v>
@@ -4921,22 +4821,22 @@
     </row>
     <row r="25" spans="1:10">
       <c r="A25" s="3" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="D25" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G25" s="3" t="s">
         <v>10</v>
@@ -4953,22 +4853,22 @@
     </row>
     <row r="26" spans="1:10">
       <c r="A26" s="2" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G26" s="2" t="s">
         <v>10</v>
@@ -4985,22 +4885,22 @@
     </row>
     <row r="27" spans="1:10">
       <c r="A27" s="3" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="D27" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G27" s="3" t="s">
         <v>10</v>
@@ -5017,22 +4917,22 @@
     </row>
     <row r="28" spans="1:10">
       <c r="A28" s="2" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G28" s="2" t="s">
         <v>10</v>
@@ -5049,22 +4949,22 @@
     </row>
     <row r="29" spans="1:10">
       <c r="A29" s="3" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="D29" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G29" s="3" t="s">
         <v>10</v>
@@ -5081,22 +4981,22 @@
     </row>
     <row r="30" spans="1:10">
       <c r="A30" s="2" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G30" s="2" t="s">
         <v>10</v>
@@ -5113,22 +5013,22 @@
     </row>
     <row r="31" spans="1:10">
       <c r="A31" s="3" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="D31" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G31" s="3" t="s">
         <v>10</v>
@@ -5145,22 +5045,22 @@
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="2" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>87</v>
+        <v>191</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G32" s="2" t="s">
         <v>10</v>
@@ -5169,7 +5069,7 @@
         <v>10</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>10</v>
+        <v>192</v>
       </c>
       <c r="J32" s="2" t="s">
         <v>10</v>
@@ -5177,22 +5077,22 @@
     </row>
     <row r="33" spans="1:10">
       <c r="A33" s="3" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="D33" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G33" s="3" t="s">
         <v>10</v>
@@ -5209,22 +5109,22 @@
     </row>
     <row r="34" spans="1:10">
       <c r="A34" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="C34" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="B34" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>201</v>
-      </c>
       <c r="D34" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G34" s="2" t="s">
         <v>10</v>
@@ -5241,22 +5141,22 @@
     </row>
     <row r="35" spans="1:10">
       <c r="A35" s="3" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="D35" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G35" s="3" t="s">
         <v>10</v>
@@ -5273,22 +5173,22 @@
     </row>
     <row r="36" spans="1:10">
       <c r="A36" s="2" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G36" s="2" t="s">
         <v>10</v>
@@ -5305,22 +5205,22 @@
     </row>
     <row r="37" spans="1:10">
       <c r="A37" s="3" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="D37" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G37" s="3" t="s">
         <v>10</v>
@@ -5329,7 +5229,7 @@
         <v>10</v>
       </c>
       <c r="I37" s="3" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="J37" s="3" t="s">
         <v>10</v>
@@ -5337,22 +5237,22 @@
     </row>
     <row r="38" spans="1:10">
       <c r="A38" s="2" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G38" s="2" t="s">
         <v>10</v>
@@ -5369,22 +5269,22 @@
     </row>
     <row r="39" spans="1:10">
       <c r="A39" s="3" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="D39" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G39" s="3" t="s">
         <v>10</v>
@@ -5401,22 +5301,22 @@
     </row>
     <row r="40" spans="1:10">
       <c r="A40" s="2" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="D40" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G40" s="2" t="s">
         <v>10</v>
@@ -5433,22 +5333,22 @@
     </row>
     <row r="41" spans="1:10">
       <c r="A41" s="3" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="D41" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G41" s="3" t="s">
         <v>10</v>
@@ -5465,22 +5365,22 @@
     </row>
     <row r="42" spans="1:10">
       <c r="A42" s="2" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G42" s="2" t="s">
         <v>10</v>
@@ -5497,22 +5397,22 @@
     </row>
     <row r="43" spans="1:10">
       <c r="A43" s="3" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="D43" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G43" s="3" t="s">
         <v>10</v>
@@ -5529,22 +5429,22 @@
     </row>
     <row r="44" spans="1:10">
       <c r="A44" s="2" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G44" s="2" t="s">
         <v>10</v>
@@ -5561,22 +5461,22 @@
     </row>
     <row r="45" spans="1:10">
       <c r="A45" s="3" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="D45" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G45" s="3" t="s">
         <v>10</v>
@@ -5593,22 +5493,22 @@
     </row>
     <row r="46" spans="1:10">
       <c r="A46" s="2" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="D46" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G46" s="2" t="s">
         <v>10</v>
@@ -5625,22 +5525,22 @@
     </row>
     <row r="47" spans="1:10">
       <c r="A47" s="3" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="D47" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F47" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G47" s="3" t="s">
         <v>10</v>
@@ -5657,22 +5557,22 @@
     </row>
     <row r="48" spans="1:10">
       <c r="A48" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="D48" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G48" s="2" t="s">
         <v>10</v>
@@ -5689,22 +5589,22 @@
     </row>
     <row r="49" spans="1:10">
       <c r="A49" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="C49" s="3" t="s">
         <v>229</v>
       </c>
-      <c r="B49" s="3" t="s">
-        <v>232</v>
-      </c>
-      <c r="C49" s="3" t="s">
-        <v>233</v>
-      </c>
       <c r="D49" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F49" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G49" s="3" t="s">
         <v>10</v>
@@ -5713,7 +5613,7 @@
         <v>10</v>
       </c>
       <c r="I49" s="3" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="J49" s="3" t="s">
         <v>10</v>
@@ -5721,22 +5621,22 @@
     </row>
     <row r="50" spans="1:10">
       <c r="A50" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="D50" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G50" s="2" t="s">
         <v>10</v>
@@ -5753,22 +5653,22 @@
     </row>
     <row r="51" spans="1:10">
       <c r="A51" s="3" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="D51" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G51" s="3" t="s">
         <v>10</v>
@@ -5785,22 +5685,22 @@
     </row>
     <row r="52" spans="1:10">
       <c r="A52" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="D52" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G52" s="2" t="s">
         <v>10</v>
@@ -5817,22 +5717,22 @@
     </row>
     <row r="53" spans="1:10">
       <c r="A53" s="3" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="D53" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F53" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G53" s="3" t="s">
         <v>10</v>
@@ -5849,22 +5749,22 @@
     </row>
     <row r="54" spans="1:10">
       <c r="A54" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="D54" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G54" s="2" t="s">
         <v>10</v>
@@ -5881,22 +5781,22 @@
     </row>
     <row r="55" spans="1:10">
       <c r="A55" s="3" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="D55" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F55" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G55" s="3" t="s">
         <v>10</v>
@@ -5913,22 +5813,22 @@
     </row>
     <row r="56" spans="1:10">
       <c r="A56" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="D56" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G56" s="2" t="s">
         <v>10</v>
@@ -5945,22 +5845,22 @@
     </row>
     <row r="57" spans="1:10">
       <c r="A57" s="3" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="D57" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F57" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G57" s="3" t="s">
         <v>10</v>
@@ -5977,22 +5877,22 @@
     </row>
     <row r="58" spans="1:10">
       <c r="A58" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="C58" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="B58" s="2" t="s">
-        <v>252</v>
-      </c>
-      <c r="C58" s="2" t="s">
-        <v>253</v>
-      </c>
       <c r="D58" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G58" s="2" t="s">
         <v>10</v>
@@ -6009,22 +5909,22 @@
     </row>
     <row r="59" spans="1:10">
       <c r="A59" s="3" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="D59" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="F59" s="3" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="G59" s="3" t="s">
         <v>10</v>
@@ -6041,22 +5941,22 @@
     </row>
     <row r="60" spans="1:10">
       <c r="A60" s="2" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="D60" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G60" s="2" t="s">
         <v>10</v>
@@ -6065,7 +5965,7 @@
         <v>10</v>
       </c>
       <c r="I60" s="2" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="J60" s="2" t="s">
         <v>10</v>
@@ -6073,22 +5973,22 @@
     </row>
     <row r="61" spans="1:10">
       <c r="A61" s="3" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="D61" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E61" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F61" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G61" s="3" t="s">
         <v>10</v>
@@ -6105,22 +6005,22 @@
     </row>
     <row r="62" spans="1:10">
       <c r="A62" s="2" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="D62" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F62" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G62" s="2" t="s">
         <v>10</v>
@@ -6137,22 +6037,22 @@
     </row>
     <row r="63" spans="1:10">
       <c r="A63" s="3" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="D63" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E63" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F63" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G63" s="3" t="s">
         <v>10</v>
@@ -6169,22 +6069,22 @@
     </row>
     <row r="64" spans="1:10">
       <c r="A64" s="2" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="B64" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="D64" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F64" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G64" s="2" t="s">
         <v>10</v>
@@ -6193,30 +6093,30 @@
         <v>10</v>
       </c>
       <c r="I64" s="2" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="J64" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="65" spans="1:10">
       <c r="A65" s="3" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="B65" s="3" t="s">
         <v>10</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="D65" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E65" s="3" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="F65" s="3" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="G65" s="3" t="s">
         <v>10</v>
@@ -6225,30 +6125,30 @@
         <v>10</v>
       </c>
       <c r="I65" s="3" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="J65" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="66" spans="1:10">
       <c r="A66" s="2" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B66" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="D66" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F66" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G66" s="2" t="s">
         <v>10</v>
@@ -6257,30 +6157,30 @@
         <v>10</v>
       </c>
       <c r="I66" s="2" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="J66" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="67" spans="1:10">
       <c r="A67" s="3" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="B67" s="3" t="s">
         <v>10</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="D67" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E67" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F67" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G67" s="3" t="s">
         <v>10</v>
@@ -6289,30 +6189,30 @@
         <v>10</v>
       </c>
       <c r="I67" s="3" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="J67" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="68" spans="1:10">
       <c r="A68" s="2" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="B68" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="D68" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="F68" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G68" s="2" t="s">
         <v>10</v>
@@ -6321,10 +6221,10 @@
         <v>10</v>
       </c>
       <c r="I68" s="2" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="J68" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -6353,16 +6253,16 @@
   <sheetData>
     <row r="1" ht="17" spans="1:10">
       <c r="A1" s="1" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>3</v>
@@ -6385,28 +6285,28 @@
     </row>
     <row r="2" spans="1:10">
       <c r="A2" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>282</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>283</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>284</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>285</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>286</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>10</v>
@@ -6417,28 +6317,28 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" s="3" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="C3" s="3" t="s">
+        <v>280</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="H3" s="3" t="s">
         <v>284</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>285</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>288</v>
       </c>
       <c r="I3" s="3" t="s">
         <v>10</v>
@@ -6449,28 +6349,28 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" s="2" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>10</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>10</v>
@@ -6481,28 +6381,28 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="3" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>10</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G5" s="3" t="s">
         <v>10</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="I5" s="3" t="s">
         <v>10</v>
@@ -6513,28 +6413,28 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" s="2" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>10</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>10</v>
@@ -6545,28 +6445,28 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" s="3" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>10</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G7" s="3" t="s">
         <v>10</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="I7" s="3" t="s">
         <v>10</v>
@@ -6577,28 +6477,28 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="2" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>10</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>10</v>
@@ -6609,28 +6509,28 @@
     </row>
     <row r="9" spans="1:10">
       <c r="A9" s="3" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>10</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G9" s="3" t="s">
         <v>10</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="I9" s="3" t="s">
         <v>10</v>
@@ -6641,31 +6541,31 @@
     </row>
     <row r="10" spans="1:10">
       <c r="A10" s="2" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>10</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="J10" s="2" t="s">
         <v>10</v>
@@ -6673,28 +6573,28 @@
     </row>
     <row r="11" spans="1:10">
       <c r="A11" s="3" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
       <c r="C11" s="3" t="s">
+        <v>301</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="H11" s="3" t="s">
         <v>305</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>285</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="H11" s="3" t="s">
-        <v>309</v>
       </c>
       <c r="I11" s="3" t="s">
         <v>10</v>
@@ -6705,28 +6605,28 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="2" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>10</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>10</v>
@@ -6737,28 +6637,28 @@
     </row>
     <row r="13" spans="1:10">
       <c r="A13" s="3" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>10</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G13" s="3" t="s">
         <v>10</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="I13" s="3" t="s">
         <v>10</v>
@@ -6769,28 +6669,28 @@
     </row>
     <row r="14" spans="1:10">
       <c r="A14" s="2" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>10</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="I14" s="2" t="s">
         <v>10</v>
@@ -6801,28 +6701,28 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" s="3" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>10</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G15" s="3" t="s">
         <v>10</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="I15" s="3" t="s">
         <v>10</v>
@@ -6833,28 +6733,28 @@
     </row>
     <row r="16" spans="1:10">
       <c r="A16" s="2" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>10</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="I16" s="2" t="s">
         <v>10</v>
@@ -6865,28 +6765,28 @@
     </row>
     <row r="17" spans="1:10">
       <c r="A17" s="3" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>10</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G17" s="3" t="s">
         <v>10</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="I17" s="3" t="s">
         <v>10</v>
@@ -6897,31 +6797,31 @@
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="2" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>10</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="J18" s="2" t="s">
         <v>10</v>
@@ -6929,31 +6829,31 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" s="3" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>10</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G19" s="3" t="s">
         <v>10</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="J19" s="3" t="s">
         <v>10</v>
@@ -6961,28 +6861,28 @@
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="2" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D20" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H20" s="2" t="s">
         <v>330</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="G20" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="H20" s="2" t="s">
-        <v>334</v>
       </c>
       <c r="I20" s="2" t="s">
         <v>10</v>
@@ -6993,35 +6893,33 @@
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="3" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>10</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G21" s="3" t="s">
         <v>10</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="I21" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="J21" s="4" t="s">
-        <v>337</v>
-      </c>
+      <c r="J21" s="4"/>
     </row>
   </sheetData>
   <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:J21" etc:filterBottomFollowUsedRange="0">

</xml_diff>